<commit_message>
added dac, storage and transport
</commit_message>
<xml_diff>
--- a/mes_north_sea/clean_data/cost_networks/NetworkCost.xlsx
+++ b/mes_north_sea/clean_data/cost_networks/NetworkCost.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\6574114\Documents\Research\EHUB-Py_Productive\mes_north_sea\clean_data\cost_networks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maiant/PycharmProjects/Key-Infrastructure-North-Sea-CodeAndData/mes_north_sea/clean_data/cost_networks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7817143-AED4-480F-8806-4175C125F6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F427CD7C-586D-1D4E-8820-1B795AF471A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A0B038B2-1901-4BA8-93AC-5F1953A9A6DA}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" xr2:uid="{A0B038B2-1901-4BA8-93AC-5F1953A9A6DA}"/>
   </bookViews>
   <sheets>
     <sheet name="ToModel" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="139">
   <si>
     <t>Type</t>
   </si>
@@ -483,6 +483,12 @@
   </si>
   <si>
     <t>H2 Pipeline (Onshore, repurposed)</t>
+  </si>
+  <si>
+    <t>CO2_Pipeline</t>
+  </si>
+  <si>
+    <t>DEA</t>
   </si>
 </sst>
 </file>
@@ -490,12 +496,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
-    <numFmt numFmtId="44" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ _F_t_-;\-* #,##0.00\ _F_t_-;_-* &quot;-&quot;??\ _F_t_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0.0000%"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ _F_t_-;\-* #,##0.00\ _F_t_-;_-* &quot;-&quot;??\ _F_t_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="0.0000%"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="_ * #,##0.000_ ;_ * \-#,##0.000_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -612,30 +618,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="5" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Comma" xfId="5" builtinId="3"/>
@@ -882,6 +886,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -889,7 +894,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -1122,6 +1126,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1129,7 +1134,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -1362,6 +1366,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1369,7 +1374,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -1602,6 +1606,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1609,7 +1614,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -1842,6 +1846,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1849,7 +1854,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -2178,6 +2182,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2185,7 +2190,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -2514,6 +2518,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2521,7 +2526,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -2850,6 +2854,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2857,7 +2862,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -3132,6 +3136,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3139,7 +3144,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -3372,6 +3376,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3379,7 +3384,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:printSettings>
     <c:headerFooter/>
@@ -3755,9 +3759,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3795,7 +3799,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3901,7 +3905,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4043,7 +4047,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4052,165 +4056,165 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A4BAA7A-A190-40C3-8275-483C16A74E0D}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="10" width="17.85546875" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="10" width="17.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="18" width="16.42578125" customWidth="1"/>
-    <col min="19" max="19" width="75.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="60.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="59.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="51.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="50.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="51.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="58.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="31" max="32" width="65.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="34" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="50.7109375" bestFit="1" customWidth="1"/>
-    <col min="36" max="37" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="48.28515625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="55.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="49.140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="76.5703125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="72.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="16.5" customWidth="1"/>
+    <col min="19" max="19" width="75.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="60.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="50.5" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="58.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="55.1640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="58.33203125" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="65.5" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="37" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="58.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="55.5" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="49.1640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="45.83203125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="76.5" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="72.83203125" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="80" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="64.140625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="57.7109375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="51.5703125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="64.1640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="57.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="51.5" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="60" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="55.5703125" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="49.140625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="56.28515625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="49.42578125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="56.5703125" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="55.5" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="49.1640625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="56.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="49.5" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="56.5" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="73" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="91.5703125" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="65.5703125" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="77.42578125" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="63.28515625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="48.85546875" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="81.1640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="91.5" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="65.5" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="59.5" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="77.5" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="48.5" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="63.33203125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="48.83203125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="39.6640625" bestFit="1" customWidth="1"/>
     <col min="66" max="66" width="38" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="14.5" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="26" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="53.42578125" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="38.85546875" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="52.7109375" bestFit="1" customWidth="1"/>
-    <col min="78" max="79" width="46.28515625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="45.5703125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="82" max="83" width="46.28515625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="53.28515625" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="51.7109375" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="75.28515625" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="60.42578125" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="59.28515625" bestFit="1" customWidth="1"/>
-    <col min="89" max="90" width="51.140625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="50.5703125" bestFit="1" customWidth="1"/>
-    <col min="92" max="93" width="51.140625" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="58.7109375" bestFit="1" customWidth="1"/>
-    <col min="95" max="96" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="98" max="99" width="65.42578125" bestFit="1" customWidth="1"/>
-    <col min="100" max="101" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="50.7109375" bestFit="1" customWidth="1"/>
-    <col min="103" max="104" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="58.28515625" bestFit="1" customWidth="1"/>
-    <col min="106" max="106" width="48.28515625" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="55.42578125" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="49.140625" bestFit="1" customWidth="1"/>
-    <col min="109" max="109" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="76.5703125" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="72.85546875" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="27.83203125" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="53.5" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="38.83203125" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="78" max="79" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="45.5" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="42.5" bestFit="1" customWidth="1"/>
+    <col min="82" max="83" width="46.33203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="51.6640625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="75.33203125" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="60.5" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="89" max="90" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="50.5" bestFit="1" customWidth="1"/>
+    <col min="92" max="93" width="51.1640625" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="58.6640625" bestFit="1" customWidth="1"/>
+    <col min="95" max="96" width="55.1640625" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="58.33203125" bestFit="1" customWidth="1"/>
+    <col min="98" max="99" width="65.5" bestFit="1" customWidth="1"/>
+    <col min="100" max="101" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="103" max="104" width="51.33203125" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="58.33203125" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="55.5" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="49.1640625" bestFit="1" customWidth="1"/>
+    <col min="109" max="109" width="45.83203125" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="76.5" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="72.83203125" bestFit="1" customWidth="1"/>
     <col min="112" max="112" width="80" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="64.140625" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="57.7109375" bestFit="1" customWidth="1"/>
-    <col min="115" max="115" width="51.5703125" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="64.1640625" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="57.6640625" bestFit="1" customWidth="1"/>
+    <col min="115" max="115" width="51.5" bestFit="1" customWidth="1"/>
     <col min="116" max="116" width="60" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="55.5703125" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="49.140625" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="56.28515625" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="49.42578125" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="56.5703125" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="55.5" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="49.1640625" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="56.33203125" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="49.5" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="56.5" bestFit="1" customWidth="1"/>
     <col min="122" max="122" width="73" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="91.5703125" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="65.5703125" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="127" max="127" width="77.42578125" bestFit="1" customWidth="1"/>
-    <col min="128" max="128" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="63.28515625" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="81.1640625" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="91.5" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="65.5" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="59.5" bestFit="1" customWidth="1"/>
+    <col min="127" max="127" width="77.5" bestFit="1" customWidth="1"/>
+    <col min="128" max="128" width="48.5" bestFit="1" customWidth="1"/>
+    <col min="129" max="129" width="63.33203125" bestFit="1" customWidth="1"/>
     <col min="130" max="130" width="39" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="133" max="133" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="135" max="135" width="44.140625" bestFit="1" customWidth="1"/>
-    <col min="136" max="136" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="137" max="137" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="138" max="138" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="139" max="139" width="47.140625" bestFit="1" customWidth="1"/>
-    <col min="140" max="140" width="57.28515625" bestFit="1" customWidth="1"/>
-    <col min="141" max="141" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="71.5703125" bestFit="1" customWidth="1"/>
-    <col min="143" max="143" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="32.5703125" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="70.5703125" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="133" max="133" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="135" max="135" width="44.1640625" bestFit="1" customWidth="1"/>
+    <col min="136" max="136" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="137" max="137" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="138" max="138" width="46.83203125" bestFit="1" customWidth="1"/>
+    <col min="139" max="139" width="47.1640625" bestFit="1" customWidth="1"/>
+    <col min="140" max="140" width="57.33203125" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="30.83203125" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="71.5" bestFit="1" customWidth="1"/>
+    <col min="143" max="143" width="45.83203125" bestFit="1" customWidth="1"/>
+    <col min="144" max="144" width="32.5" bestFit="1" customWidth="1"/>
+    <col min="145" max="145" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="146" max="146" width="70.5" bestFit="1" customWidth="1"/>
     <col min="147" max="147" width="45" bestFit="1" customWidth="1"/>
     <col min="148" max="148" width="31" bestFit="1" customWidth="1"/>
-    <col min="149" max="149" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="151" max="151" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="149" max="149" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="150" max="150" width="55.1640625" bestFit="1" customWidth="1"/>
+    <col min="151" max="151" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="152" max="152" width="61" bestFit="1" customWidth="1"/>
-    <col min="153" max="153" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="154" max="155" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="156" max="156" width="37.5703125" bestFit="1" customWidth="1"/>
-    <col min="157" max="157" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="153" max="153" width="42.1640625" bestFit="1" customWidth="1"/>
+    <col min="154" max="155" width="34.5" bestFit="1" customWidth="1"/>
+    <col min="156" max="156" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="157" max="157" width="33.83203125" bestFit="1" customWidth="1"/>
     <col min="158" max="158" width="24" bestFit="1" customWidth="1"/>
-    <col min="159" max="161" width="36.42578125" bestFit="1" customWidth="1"/>
-    <col min="162" max="162" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="163" max="163" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="165" max="165" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="166" max="168" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="170" max="171" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="172" max="173" width="65.42578125" bestFit="1" customWidth="1"/>
-    <col min="174" max="174" width="47.85546875" bestFit="1" customWidth="1"/>
-    <col min="175" max="175" width="42.85546875" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="47.85546875" bestFit="1" customWidth="1"/>
+    <col min="159" max="161" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="162" max="162" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="163" max="163" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="164" max="164" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="166" max="168" width="39.83203125" bestFit="1" customWidth="1"/>
+    <col min="169" max="169" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="170" max="171" width="39.83203125" bestFit="1" customWidth="1"/>
+    <col min="172" max="173" width="65.5" bestFit="1" customWidth="1"/>
+    <col min="174" max="174" width="47.83203125" bestFit="1" customWidth="1"/>
+    <col min="175" max="175" width="42.83203125" bestFit="1" customWidth="1"/>
+    <col min="176" max="176" width="47.83203125" bestFit="1" customWidth="1"/>
     <col min="177" max="177" width="45" bestFit="1" customWidth="1"/>
     <col min="178" max="178" width="40" bestFit="1" customWidth="1"/>
     <col min="179" max="179" width="45" bestFit="1" customWidth="1"/>
-    <col min="180" max="180" width="52.28515625" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="182" max="182" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="180" max="180" width="52.33203125" bestFit="1" customWidth="1"/>
+    <col min="181" max="181" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>17</v>
       </c>
@@ -4236,7 +4240,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -4295,7 +4299,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -4308,18 +4312,18 @@
       <c r="D3">
         <v>0</v>
       </c>
-      <c r="E3" s="11">
-        <v>0</v>
-      </c>
-      <c r="F3" s="11">
+      <c r="E3" s="10">
+        <v>0</v>
+      </c>
+      <c r="F3" s="10">
         <f>ROUND(C3*$S3,0)</f>
         <v>43695</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="10">
         <f>ROUND(D3*$S3,0)</f>
         <v>0</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <f>ROUND(B3*$S3,0)</f>
         <v>372</v>
       </c>
@@ -4353,7 +4357,7 @@
         <v>1.1261624192640001</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -4366,18 +4370,18 @@
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="11">
-        <v>0</v>
-      </c>
-      <c r="F4" s="11">
+      <c r="E4" s="10">
+        <v>0</v>
+      </c>
+      <c r="F4" s="10">
         <f t="shared" ref="F4:F5" si="0">ROUND(C4*$S4,0)</f>
         <v>136266</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <f t="shared" ref="G4:G5" si="1">ROUND(D4*$S4,0)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <f t="shared" ref="H4:H5" si="2">ROUND(B4*$S4,0)</f>
         <v>270</v>
       </c>
@@ -4411,7 +4415,7 @@
         <v>1.1261624192640001</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -4426,18 +4430,18 @@
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="11">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11">
+      <c r="E5" s="10">
+        <v>0</v>
+      </c>
+      <c r="F5" s="10">
         <f t="shared" si="0"/>
         <v>136265653</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <f t="shared" si="2"/>
         <v>270279</v>
       </c>
@@ -4471,23 +4475,23 @@
         <v>1.1261624192640001</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>130</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <f>'H2'!B16</f>
         <v>337045654.09746808</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="10">
         <f>'H2'!C16</f>
         <v>-33086.598776513507</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <f>'H2'!D16</f>
         <v>0</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <f>'H2'!E16</f>
         <v>513.99989612008517</v>
       </c>
@@ -4514,23 +4518,23 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>131</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="10">
         <f>'H2'!B15</f>
         <v>198262149.46909887</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="10">
         <f>'H2'!C15</f>
         <v>-19462.705162655006</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <f>'H2'!D15</f>
         <v>0</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <f>'H2'!E15</f>
         <v>302.35288007063832</v>
       </c>
@@ -4557,23 +4561,23 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>132</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <f>'H2'!B14</f>
         <v>39567835.104559466</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="10">
         <f>'H2'!C14</f>
         <v>-3840.2806153825454</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <f>'H2'!D14</f>
         <v>0</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <f>'H2'!E14</f>
         <v>92.540894220283576</v>
       </c>
@@ -4598,6 +4602,44 @@
       </c>
       <c r="O8" t="s">
         <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>33000</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>50</v>
+      </c>
+      <c r="L9">
+        <v>6.0999999999999999E-2</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>2040</v>
+      </c>
+      <c r="O9" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -4612,13 +4654,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{019F240E-8503-41E7-B90B-86BA10EB15EF}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:S20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>109</v>
       </c>
@@ -4626,7 +4668,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>67</v>
       </c>
@@ -4679,7 +4721,7 @@
         <v>gamma1 &amp; [kEUR] &amp; 0 &amp; 0 &amp; 337045.65 &amp; 198262.15 &amp; 39567.84\\</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>68</v>
       </c>
@@ -4708,23 +4750,23 @@
         <v>112</v>
       </c>
       <c r="K3">
-        <f t="shared" ref="K3:K10" si="1">ROUND(C3,2)</f>
+        <f t="shared" ref="K3:K9" si="1">ROUND(C3,2)</f>
         <v>43.7</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:L10" si="2">ROUND(D3,2)</f>
+        <f t="shared" ref="L3:L9" si="2">ROUND(D3,2)</f>
         <v>68.13</v>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M10" si="3">ROUND(E3,2)</f>
+        <f t="shared" ref="M3:M9" si="3">ROUND(E3,2)</f>
         <v>-33.090000000000003</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N10" si="4">ROUND(F3,2)</f>
+        <f t="shared" ref="N3:N9" si="4">ROUND(F3,2)</f>
         <v>-19.46</v>
       </c>
       <c r="O3">
-        <f t="shared" ref="O3:O10" si="5">ROUND(G3,2)</f>
+        <f t="shared" ref="O3:O9" si="5">ROUND(G3,2)</f>
         <v>-3.84</v>
       </c>
       <c r="S3" t="str">
@@ -4732,7 +4774,7 @@
         <v>gamma2 &amp; [kEUR/MW] &amp; 43.7 &amp; 68.13 &amp; -33.09 &amp; -19.46 &amp; -3.84\\</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -4785,7 +4827,7 @@
         <v>gamma3 &amp; [kEUR/km] &amp; 0 &amp; 0 &amp; 0 &amp; 0 &amp; 0\\</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -4838,7 +4880,7 @@
         <v>gamma4 &amp; [kEUR/km/MW] &amp; 0.37 &amp; 0.14 &amp; 0.51 &amp; 0.3 &amp; 0.09\\</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -4891,7 +4933,7 @@
         <v>rated power &amp; [MW] &amp; 1 &amp; 2000 &amp; 1 &amp; 1 &amp; 1\\</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -4944,7 +4986,7 @@
         <v>Lifetime &amp; [a] &amp; 40 &amp; 40 &amp; 50 &amp; 50 &amp; 50\\</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -4997,7 +5039,7 @@
         <v>OPEX Fixed &amp; [\% annual CAPEX] &amp; 0.04 &amp; 0.04 &amp; 0.04 &amp; 0.04 &amp; 0.04\\</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -5050,7 +5092,7 @@
         <v>OPEX Variable &amp; [EUR/MWh] &amp; 0 &amp; 0 &amp; 0 &amp; 0 &amp; 0\\</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -5092,91 +5134,91 @@
         <v>Source &amp;  &amp; \cite{Zappa2019} &amp; \cite{Zappa2019} &amp; \cite{EHB2022} &amp; \cite{EHB2022} &amp; \cite{EHB2022}\\</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;B14&amp;"}}"</f>
+        <f t="shared" ref="B12:J12" si="7">"\multicolumn{1}{c}{\makecell{"&amp;B14&amp;"}}"</f>
         <v>\multicolumn{1}{c}{\makecell{gamma1}}</v>
       </c>
       <c r="C12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;C14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{gamma2}}</v>
       </c>
       <c r="D12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;D14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{gamma3}}</v>
       </c>
       <c r="E12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;E14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{gamma4}}</v>
       </c>
       <c r="F12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;F14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{rated power}}</v>
       </c>
       <c r="G12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;G14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{Lifetime}}</v>
       </c>
       <c r="H12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;H14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{OPEX Fixed}}</v>
       </c>
       <c r="I12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;I14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{OPEX Variable}}</v>
       </c>
       <c r="J12" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;J14&amp;"}}"</f>
+        <f t="shared" si="7"/>
         <v>\multicolumn{1}{c}{\makecell{Source}}</v>
       </c>
       <c r="L12" t="str">
-        <f t="shared" ref="L12:L13" si="7">_xlfn.TEXTJOIN(" &amp; ",FALSE,A12:J12)&amp;"\\"</f>
+        <f t="shared" ref="L12:L13" si="8">_xlfn.TEXTJOIN(" &amp; ",FALSE,A12:J12)&amp;"\\"</f>
         <v xml:space="preserve"> &amp; \multicolumn{1}{c}{\makecell{gamma1}} &amp; \multicolumn{1}{c}{\makecell{gamma2}} &amp; \multicolumn{1}{c}{\makecell{gamma3}} &amp; \multicolumn{1}{c}{\makecell{gamma4}} &amp; \multicolumn{1}{c}{\makecell{rated power}} &amp; \multicolumn{1}{c}{\makecell{Lifetime}} &amp; \multicolumn{1}{c}{\makecell{OPEX Fixed}} &amp; \multicolumn{1}{c}{\makecell{OPEX Variable}} &amp; \multicolumn{1}{c}{\makecell{Source}}\\</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;B15&amp;"}}"</f>
+        <f t="shared" ref="B13:J13" si="9">"\multicolumn{1}{c}{\makecell{"&amp;B15&amp;"}}"</f>
         <v>\multicolumn{1}{c}{\makecell{[kEUR]}}</v>
       </c>
       <c r="C13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;C15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[kEUR/MW]}}</v>
       </c>
       <c r="D13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;D15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[kEUR/km]}}</v>
       </c>
       <c r="E13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;E15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[kEUR/km/MW]}}</v>
       </c>
       <c r="F13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;F15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[MW]}}</v>
       </c>
       <c r="G13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;G15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[a]}}</v>
       </c>
       <c r="H13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;H15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[\% annual CAPEX]}}</v>
       </c>
       <c r="I13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;I15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{[EUR/MWh]}}</v>
       </c>
       <c r="J13" t="str">
-        <f>"\multicolumn{1}{c}{\makecell{"&amp;J15&amp;"}}"</f>
+        <f t="shared" si="9"/>
         <v>\multicolumn{1}{c}{\makecell{0}}</v>
       </c>
       <c r="L13" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v xml:space="preserve"> &amp; \multicolumn{1}{c}{\makecell{[kEUR]}} &amp; \multicolumn{1}{c}{\makecell{[kEUR/MW]}} &amp; \multicolumn{1}{c}{\makecell{[kEUR/km]}} &amp; \multicolumn{1}{c}{\makecell{[kEUR/km/MW]}} &amp; \multicolumn{1}{c}{\makecell{[MW]}} &amp; \multicolumn{1}{c}{\makecell{[a]}} &amp; \multicolumn{1}{c}{\makecell{[\% annual CAPEX]}} &amp; \multicolumn{1}{c}{\makecell{[EUR/MWh]}} &amp; \multicolumn{1}{c}{\makecell{0}}\\</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B14" t="str" cm="1">
         <f t="array" ref="B14:J20">TRANSPOSE(I2:O10)</f>
         <v>gamma1</v>
@@ -5210,7 +5252,7 @@
         <v xml:space="preserve"> &amp; gamma1 &amp; gamma2 &amp; gamma3 &amp; gamma4 &amp; rated power &amp; Lifetime &amp; OPEX Fixed &amp; OPEX Variable &amp; Source\\</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="B15" t="str">
         <v>[kEUR]</v>
       </c>
@@ -5239,11 +5281,11 @@
         <v>0</v>
       </c>
       <c r="L15" t="str">
-        <f t="shared" ref="L15:L20" si="8">_xlfn.TEXTJOIN(" &amp; ",FALSE,A15:J15)&amp;"\\"</f>
+        <f t="shared" ref="L15:L20" si="10">_xlfn.TEXTJOIN(" &amp; ",FALSE,A15:J15)&amp;"\\"</f>
         <v xml:space="preserve"> &amp; [kEUR] &amp; [kEUR/MW] &amp; [kEUR/km] &amp; [kEUR/km/MW] &amp; [MW] &amp; [a] &amp; [\% annual CAPEX] &amp; [EUR/MWh] &amp; 0\\</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>109</v>
       </c>
@@ -5275,11 +5317,11 @@
         <v>\cite{Zappa2019}</v>
       </c>
       <c r="L16" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>Electricity AC &amp; 0 &amp; 43.7 &amp; 0 &amp; 0.37 &amp; 1 &amp; 40 &amp; 0.04 &amp; 0 &amp; \cite{Zappa2019}\\</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>110</v>
       </c>
@@ -5311,11 +5353,11 @@
         <v>\cite{Zappa2019}</v>
       </c>
       <c r="L17" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>Electricity DC &amp; 0 &amp; 68.13 &amp; 0 &amp; 0.14 &amp; 2000 &amp; 40 &amp; 0.04 &amp; 0 &amp; \cite{Zappa2019}\\</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>134</v>
       </c>
@@ -5347,11 +5389,11 @@
         <v>\cite{EHB2022}</v>
       </c>
       <c r="L18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>H2 Pipeline (Offshore) &amp; 337045.65 &amp; -33.09 &amp; 0 &amp; 0.51 &amp; 1 &amp; 50 &amp; 0.04 &amp; 0 &amp; \cite{EHB2022}\\</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>135</v>
       </c>
@@ -5383,11 +5425,11 @@
         <v>\cite{EHB2022}</v>
       </c>
       <c r="L19" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>H2 Pipeline (Onshore, new) &amp; 198262.15 &amp; -19.46 &amp; 0 &amp; 0.3 &amp; 1 &amp; 50 &amp; 0.04 &amp; 0 &amp; \cite{EHB2022}\\</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>136</v>
       </c>
@@ -5419,7 +5461,7 @@
         <v>\cite{EHB2022}</v>
       </c>
       <c r="L20" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>H2 Pipeline (Onshore, repurposed) &amp; 39567.84 &amp; -3.84 &amp; 0 &amp; 0.09 &amp; 1 &amp; 50 &amp; 0.04 &amp; 0 &amp; \cite{EHB2022}\\</v>
       </c>
     </row>
@@ -5432,16 +5474,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A83D4304-D793-4A46-9E41-9D5D2FD6D4F2}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI119"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -5461,7 +5503,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>62</v>
       </c>
@@ -5472,12 +5514,12 @@
         <f>(B14+C14*$L$1+E14*$N$1*$L$1)*10^-6</f>
         <v>128.7785890909866</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="12">
         <f>K2/$L$1/$N$1/1000*10^6</f>
         <v>9.9366195286255093E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>120</v>
       </c>
@@ -5488,16 +5530,16 @@
         <f>(B15+C15*$L$1+E15*$N$1*$L$1)*10^-6</f>
         <v>434.40984073940609</v>
       </c>
-      <c r="L3" s="13">
+      <c r="L3" s="11">
         <f>K2/K3</f>
         <v>0.29644491679054374</v>
       </c>
-      <c r="M3" s="14">
+      <c r="M3" s="12">
         <f t="shared" ref="M3:M4" si="0">K3/$L$1/$N$1/1000*10^6</f>
         <v>0.33519277834830713</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -5517,16 +5559,16 @@
         <f>(B16+C16*$L$1+E16*$N$1*$L$1)*10^-6</f>
         <v>738.49672925699042</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4">
         <f>K4/K3</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="12">
         <f t="shared" si="0"/>
         <v>0.56982772319212227</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -5544,7 +5586,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -5569,7 +5611,7 @@
         <v>518.4</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -5587,7 +5629,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -5605,7 +5647,7 @@
         <v>2.52</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>65</v>
       </c>
@@ -5623,7 +5665,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -5641,7 +5683,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C12" t="s">
         <v>121</v>
       </c>
@@ -5652,7 +5694,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>66</v>
       </c>
@@ -5669,70 +5711,68 @@
         <v>104</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <f>R36*10^6</f>
         <v>39567835.104559466</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="10">
         <f>R38*10^6</f>
         <v>-3840.2806153825454</v>
       </c>
-      <c r="D14" s="11">
-        <v>0</v>
-      </c>
-      <c r="E14" s="11">
+      <c r="D14" s="10">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10">
         <f>R37*10^6</f>
         <v>92.540894220283576</v>
       </c>
-      <c r="F14" s="12"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>1</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <f>AB36*10^6</f>
         <v>198262149.46909887</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <f>AB38*10^6</f>
         <v>-19462.705162655006</v>
       </c>
-      <c r="D15" s="11">
-        <v>0</v>
-      </c>
-      <c r="E15" s="11">
+      <c r="D15" s="10">
+        <v>0</v>
+      </c>
+      <c r="E15" s="10">
         <f>AB37*10^6</f>
         <v>302.35288007063832</v>
       </c>
-      <c r="F15" s="12"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>125</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="10">
         <f>B15*1.7</f>
         <v>337045654.09746808</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="10">
         <f>C15*1.7</f>
         <v>-33086.598776513507</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="10">
         <f>D15*1.7</f>
         <v>0</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="10">
         <f>E15*1.7</f>
         <v>513.99989612008517</v>
       </c>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -5740,7 +5780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -5772,7 +5812,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:32" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>50</v>
       </c>
@@ -5783,11 +5823,11 @@
       <c r="C21">
         <v>13000</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <f>($C$5+$D$5)*A21*10^6</f>
         <v>56000000.000000007</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="10">
         <f>B21*$R$37*1000000+C21*$R$38*1000000+$R$36*1000000</f>
         <v>49795768.347770706</v>
       </c>
@@ -5810,7 +5850,7 @@
         <v>141.77635440049869</v>
       </c>
     </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>100</v>
       </c>
@@ -5821,11 +5861,11 @@
       <c r="C22">
         <v>13000</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="10">
         <f t="shared" ref="D22:D40" si="3">($C$5+$D$5)*A22*10^6</f>
         <v>112000000.00000001</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="10">
         <f t="shared" ref="E22:E40" si="4">B22*$R$37*1000000+C22*$R$38*1000000+$R$36*1000000</f>
         <v>109947349.59095503</v>
       </c>
@@ -5847,16 +5887,16 @@
         <f t="shared" si="2"/>
         <v>338.30572644641359</v>
       </c>
-      <c r="Q22" s="10" t="s">
+      <c r="Q22" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="R22" s="10"/>
-      <c r="AA22" s="10" t="s">
+      <c r="R22" s="9"/>
+      <c r="AA22" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="AB22" s="10"/>
-    </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AB22" s="9"/>
+    </row>
+    <row r="23" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>150</v>
       </c>
@@ -5867,11 +5907,11 @@
       <c r="C23">
         <v>13000</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <f t="shared" si="3"/>
         <v>168000000.00000003</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="10">
         <f t="shared" si="4"/>
         <v>170098930.83413935</v>
       </c>
@@ -5893,20 +5933,20 @@
         <f t="shared" si="2"/>
         <v>534.83509849232848</v>
       </c>
-      <c r="Q23" s="7" t="s">
+      <c r="Q23" t="s">
         <v>76</v>
       </c>
-      <c r="R23" s="7">
+      <c r="R23">
         <v>0.97977577700084184</v>
       </c>
-      <c r="AA23" s="7" t="s">
+      <c r="AA23" t="s">
         <v>76</v>
       </c>
-      <c r="AB23" s="7">
+      <c r="AB23">
         <v>0.93855775701874167</v>
       </c>
     </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>200</v>
       </c>
@@ -5917,11 +5957,11 @@
       <c r="C24">
         <v>13000</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="10">
         <f t="shared" si="3"/>
         <v>224000000.00000003</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="10">
         <f t="shared" si="4"/>
         <v>230250512.07732368</v>
       </c>
@@ -5943,20 +5983,20 @@
         <f t="shared" si="2"/>
         <v>731.36447053824338</v>
       </c>
-      <c r="Q24" s="7" t="s">
+      <c r="Q24" t="s">
         <v>77</v>
       </c>
-      <c r="R24" s="7">
+      <c r="R24">
         <v>0.95996057319760342</v>
       </c>
-      <c r="AA24" s="7" t="s">
+      <c r="AA24" t="s">
         <v>77</v>
       </c>
-      <c r="AB24" s="7">
+      <c r="AB24">
         <v>0.88089066326005128</v>
       </c>
     </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>250</v>
       </c>
@@ -5967,11 +6007,11 @@
       <c r="C25">
         <v>13000</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <f t="shared" si="3"/>
         <v>280000000</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="10">
         <f t="shared" si="4"/>
         <v>290402093.32050794</v>
       </c>
@@ -5993,20 +6033,20 @@
         <f t="shared" si="2"/>
         <v>927.89384258415828</v>
       </c>
-      <c r="Q25" s="7" t="s">
+      <c r="Q25" t="s">
         <v>78</v>
       </c>
-      <c r="R25" s="7">
+      <c r="R25">
         <v>0.95106292279707083</v>
       </c>
-      <c r="AA25" s="7" t="s">
+      <c r="AA25" t="s">
         <v>78</v>
       </c>
-      <c r="AB25" s="7">
+      <c r="AB25">
         <v>0.85442192176228504</v>
       </c>
     </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>300</v>
       </c>
@@ -6017,11 +6057,11 @@
       <c r="C26">
         <v>13000</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="10">
         <f t="shared" si="3"/>
         <v>336000000.00000006</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="10">
         <f t="shared" si="4"/>
         <v>350553674.56369239</v>
       </c>
@@ -6043,20 +6083,20 @@
         <f t="shared" si="2"/>
         <v>1124.4232146300733</v>
       </c>
-      <c r="Q26" s="7" t="s">
+      <c r="Q26" t="s">
         <v>79</v>
       </c>
-      <c r="R26" s="7">
+      <c r="R26">
         <v>13.307416758100223</v>
       </c>
-      <c r="AA26" s="7" t="s">
+      <c r="AA26" t="s">
         <v>79</v>
       </c>
-      <c r="AB26" s="7">
+      <c r="AB26">
         <v>69.201448774718187</v>
       </c>
     </row>
-    <row r="27" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:32" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>350</v>
       </c>
@@ -6067,11 +6107,11 @@
       <c r="C27">
         <v>13000</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="10">
         <f t="shared" si="3"/>
         <v>392000000.00000006</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="10">
         <f t="shared" si="4"/>
         <v>410705255.8068766</v>
       </c>
@@ -6093,20 +6133,20 @@
         <f t="shared" si="2"/>
         <v>1320.9525866759882</v>
       </c>
-      <c r="Q27" s="8" t="s">
+      <c r="Q27" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="R27" s="8">
+      <c r="R27" s="7">
         <v>12</v>
       </c>
-      <c r="AA27" s="8" t="s">
+      <c r="AA27" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="AB27" s="8">
+      <c r="AB27" s="7">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>400</v>
       </c>
@@ -6117,11 +6157,11 @@
       <c r="C28">
         <v>13000</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="10">
         <f t="shared" si="3"/>
         <v>448000000.00000006</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28" s="10">
         <f t="shared" si="4"/>
         <v>470856837.05006105</v>
       </c>
@@ -6144,7 +6184,7 @@
         <v>1517.4819587219031</v>
       </c>
     </row>
-    <row r="29" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:32" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>450</v>
       </c>
@@ -6155,11 +6195,11 @@
       <c r="C29">
         <v>13000</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="10">
         <f t="shared" si="3"/>
         <v>504000000.00000006</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="10">
         <f t="shared" si="4"/>
         <v>531008418.29324526</v>
       </c>
@@ -6188,7 +6228,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>500</v>
       </c>
@@ -6199,11 +6239,11 @@
       <c r="C30">
         <v>13000</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="10">
         <f t="shared" si="3"/>
         <v>560000000</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="10">
         <f t="shared" si="4"/>
         <v>591159999.53642952</v>
       </c>
@@ -6225,40 +6265,40 @@
         <f t="shared" si="2"/>
         <v>1910.5407028137329</v>
       </c>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="9" t="s">
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="S30" s="9" t="s">
+      <c r="S30" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="T30" s="9" t="s">
+      <c r="T30" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="U30" s="9" t="s">
+      <c r="U30" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="V30" s="9" t="s">
+      <c r="V30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="AA30" s="9"/>
-      <c r="AB30" s="9" t="s">
+      <c r="AA30" s="8"/>
+      <c r="AB30" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="AC30" s="9" t="s">
+      <c r="AC30" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="AD30" s="9" t="s">
+      <c r="AD30" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="AE30" s="9" t="s">
+      <c r="AE30" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="AF30" s="9" t="s">
+      <c r="AF30" s="8" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>550</v>
       </c>
@@ -6269,11 +6309,11 @@
       <c r="C31">
         <v>13000</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="10">
         <f t="shared" si="3"/>
         <v>616000000.00000012</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="10">
         <f t="shared" si="4"/>
         <v>651311580.77961397</v>
       </c>
@@ -6295,44 +6335,44 @@
         <f t="shared" si="2"/>
         <v>2107.0700748596478</v>
       </c>
-      <c r="Q31" s="7" t="s">
+      <c r="Q31" t="s">
         <v>82</v>
       </c>
-      <c r="R31" s="7">
+      <c r="R31">
         <v>2</v>
       </c>
-      <c r="S31" s="7">
+      <c r="S31">
         <v>38211.630599702788</v>
       </c>
-      <c r="T31" s="7">
+      <c r="T31">
         <v>19105.815299851394</v>
       </c>
-      <c r="U31" s="7">
+      <c r="U31">
         <v>107.88922130949798</v>
       </c>
-      <c r="V31" s="7">
+      <c r="V31">
         <v>5.1427490430817188E-7</v>
       </c>
-      <c r="AA31" s="7" t="s">
+      <c r="AA31" t="s">
         <v>82</v>
       </c>
-      <c r="AB31" s="7">
+      <c r="AB31">
         <v>2</v>
       </c>
-      <c r="AC31" s="7">
+      <c r="AC31">
         <v>318749.18538732047</v>
       </c>
-      <c r="AD31" s="7">
+      <c r="AD31">
         <v>159374.59269366023</v>
       </c>
-      <c r="AE31" s="7">
+      <c r="AE31">
         <v>33.280413552506346</v>
       </c>
-      <c r="AF31" s="7">
+      <c r="AF31">
         <v>6.9463414638694794E-5</v>
       </c>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>600</v>
       </c>
@@ -6343,11 +6383,11 @@
       <c r="C32">
         <v>13000</v>
       </c>
-      <c r="D32" s="11">
+      <c r="D32" s="10">
         <f t="shared" si="3"/>
         <v>672000000.00000012</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="10">
         <f t="shared" si="4"/>
         <v>711463162.0227983</v>
       </c>
@@ -6369,36 +6409,32 @@
         <f t="shared" si="2"/>
         <v>2303.5994469055627</v>
       </c>
-      <c r="Q32" s="7" t="s">
+      <c r="Q32" t="s">
         <v>83</v>
       </c>
-      <c r="R32" s="7">
+      <c r="R32">
         <v>9</v>
       </c>
-      <c r="S32" s="7">
+      <c r="S32">
         <v>1593.7860669638997</v>
       </c>
-      <c r="T32" s="7">
+      <c r="T32">
         <v>177.08734077376664</v>
       </c>
-      <c r="U32" s="7"/>
-      <c r="V32" s="7"/>
-      <c r="AA32" s="7" t="s">
+      <c r="AA32" t="s">
         <v>83</v>
       </c>
-      <c r="AB32" s="7">
+      <c r="AB32">
         <v>9</v>
       </c>
-      <c r="AC32" s="7">
+      <c r="AC32">
         <v>43099.564612679504</v>
       </c>
-      <c r="AD32" s="7">
+      <c r="AD32">
         <v>4788.8405125199452</v>
       </c>
-      <c r="AE32" s="7"/>
-      <c r="AF32" s="7"/>
-    </row>
-    <row r="33" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="33" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>650</v>
       </c>
@@ -6409,11 +6445,11 @@
       <c r="C33">
         <v>13000</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="10">
         <f t="shared" si="3"/>
         <v>728000000.00000012</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="10">
         <f t="shared" si="4"/>
         <v>771614743.26598251</v>
       </c>
@@ -6435,32 +6471,32 @@
         <f t="shared" si="2"/>
         <v>2500.1288189514776</v>
       </c>
-      <c r="Q33" s="8" t="s">
+      <c r="Q33" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="R33" s="8">
+      <c r="R33" s="7">
         <v>11</v>
       </c>
-      <c r="S33" s="8">
+      <c r="S33" s="7">
         <v>39805.416666666686</v>
       </c>
-      <c r="T33" s="8"/>
-      <c r="U33" s="8"/>
-      <c r="V33" s="8"/>
-      <c r="AA33" s="8" t="s">
+      <c r="T33" s="7"/>
+      <c r="U33" s="7"/>
+      <c r="V33" s="7"/>
+      <c r="AA33" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="AB33" s="8">
+      <c r="AB33" s="7">
         <v>11</v>
       </c>
-      <c r="AC33" s="8">
+      <c r="AC33" s="7">
         <v>361848.75</v>
       </c>
-      <c r="AD33" s="8"/>
-      <c r="AE33" s="8"/>
-      <c r="AF33" s="8"/>
-    </row>
-    <row r="34" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AD33" s="7"/>
+      <c r="AE33" s="7"/>
+      <c r="AF33" s="7"/>
+    </row>
+    <row r="34" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>700</v>
       </c>
@@ -6471,11 +6507,11 @@
       <c r="C34">
         <v>13000</v>
       </c>
-      <c r="D34" s="11">
+      <c r="D34" s="10">
         <f t="shared" si="3"/>
         <v>784000000.00000012</v>
       </c>
-      <c r="E34" s="11">
+      <c r="E34" s="10">
         <f t="shared" si="4"/>
         <v>831766324.50916684</v>
       </c>
@@ -6498,7 +6534,7 @@
         <v>2696.6581909973925</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>750</v>
       </c>
@@ -6509,11 +6545,11 @@
       <c r="C35">
         <v>13000</v>
       </c>
-      <c r="D35" s="11">
+      <c r="D35" s="10">
         <f t="shared" si="3"/>
         <v>840000000.00000012</v>
       </c>
-      <c r="E35" s="11">
+      <c r="E35" s="10">
         <f t="shared" si="4"/>
         <v>891917905.75235128</v>
       </c>
@@ -6535,58 +6571,58 @@
         <f t="shared" si="2"/>
         <v>2893.1875630433074</v>
       </c>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9" t="s">
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="S35" s="9" t="s">
+      <c r="S35" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="T35" s="9" t="s">
+      <c r="T35" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="U35" s="9" t="s">
+      <c r="U35" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="V35" s="9" t="s">
+      <c r="V35" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="W35" s="9" t="s">
+      <c r="W35" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="X35" s="9" t="s">
+      <c r="X35" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="Y35" s="9" t="s">
+      <c r="Y35" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="AA35" s="9"/>
-      <c r="AB35" s="9" t="s">
+      <c r="AA35" s="8"/>
+      <c r="AB35" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="AC35" s="9" t="s">
+      <c r="AC35" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="AD35" s="9" t="s">
+      <c r="AD35" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="AE35" s="9" t="s">
+      <c r="AE35" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AF35" s="9" t="s">
+      <c r="AF35" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="AG35" s="9" t="s">
+      <c r="AG35" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="AH35" s="9" t="s">
+      <c r="AH35" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="AI35" s="9" t="s">
+      <c r="AI35" s="8" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>800</v>
       </c>
@@ -6597,11 +6633,11 @@
       <c r="C36">
         <v>13000</v>
       </c>
-      <c r="D36" s="11">
+      <c r="D36" s="10">
         <f t="shared" si="3"/>
         <v>896000000.00000012</v>
       </c>
-      <c r="E36" s="11">
+      <c r="E36" s="10">
         <f t="shared" si="4"/>
         <v>952069486.99553561</v>
       </c>
@@ -6623,62 +6659,62 @@
         <f t="shared" si="2"/>
         <v>3089.7169350892223</v>
       </c>
-      <c r="Q36" s="7" t="s">
+      <c r="Q36" t="s">
         <v>85</v>
       </c>
-      <c r="R36" s="7">
+      <c r="R36">
         <v>39.567835104559464</v>
       </c>
-      <c r="S36" s="7">
+      <c r="S36">
         <v>5.8986172990611365</v>
       </c>
-      <c r="T36" s="7">
+      <c r="T36">
         <v>6.707984786681676</v>
       </c>
-      <c r="U36" s="7">
+      <c r="U36">
         <v>8.7735845784733563E-5</v>
       </c>
-      <c r="V36" s="7">
+      <c r="V36">
         <v>26.22423573088291</v>
       </c>
-      <c r="W36" s="7">
+      <c r="W36">
         <v>52.911434478236018</v>
       </c>
-      <c r="X36" s="7">
+      <c r="X36">
         <v>26.22423573088291</v>
       </c>
-      <c r="Y36" s="7">
+      <c r="Y36">
         <v>52.911434478236018</v>
       </c>
-      <c r="AA36" s="7" t="s">
+      <c r="AA36" t="s">
         <v>85</v>
       </c>
-      <c r="AB36" s="7">
+      <c r="AB36">
         <v>198.26214946909886</v>
       </c>
-      <c r="AC36" s="7">
+      <c r="AC36">
         <v>32.340617443994461</v>
       </c>
-      <c r="AD36" s="7">
+      <c r="AD36">
         <v>6.1304379798078177</v>
       </c>
-      <c r="AE36" s="7">
+      <c r="AE36">
         <v>1.7275575511672468E-4</v>
       </c>
-      <c r="AF36" s="7">
+      <c r="AF36">
         <v>125.1025900688502</v>
       </c>
-      <c r="AG36" s="7">
+      <c r="AG36">
         <v>271.42170886934753</v>
       </c>
-      <c r="AH36" s="7">
+      <c r="AH36">
         <v>125.1025900688502</v>
       </c>
-      <c r="AI36" s="7">
+      <c r="AI36">
         <v>271.42170886934753</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>850</v>
       </c>
@@ -6689,11 +6725,11 @@
       <c r="C37">
         <v>13000</v>
       </c>
-      <c r="D37" s="11">
+      <c r="D37" s="10">
         <f t="shared" si="3"/>
         <v>952000000.00000012</v>
       </c>
-      <c r="E37" s="11">
+      <c r="E37" s="10">
         <f t="shared" si="4"/>
         <v>1012221068.2387198</v>
       </c>
@@ -6715,62 +6751,62 @@
         <f t="shared" si="2"/>
         <v>3286.2463071351372</v>
       </c>
-      <c r="Q37" s="7" t="s">
+      <c r="Q37" t="s">
         <v>97</v>
       </c>
-      <c r="R37" s="7">
+      <c r="R37">
         <v>9.2540894220283573E-5</v>
       </c>
-      <c r="S37" s="7">
+      <c r="S37">
         <v>8.7889923415008414E-6</v>
       </c>
-      <c r="T37" s="7">
+      <c r="T37">
         <v>10.529181346912056</v>
       </c>
-      <c r="U37" s="7">
+      <c r="U37">
         <v>2.3257765236709474E-6</v>
       </c>
-      <c r="V37" s="7">
+      <c r="V37">
         <v>7.2658812241178878E-5</v>
       </c>
-      <c r="W37" s="7">
+      <c r="W37">
         <v>1.1242297619938827E-4</v>
       </c>
-      <c r="X37" s="7">
+      <c r="X37">
         <v>7.2658812241178878E-5</v>
       </c>
-      <c r="Y37" s="7">
+      <c r="Y37">
         <v>1.1242297619938827E-4</v>
       </c>
-      <c r="AA37" s="7" t="s">
+      <c r="AA37" t="s">
         <v>97</v>
       </c>
-      <c r="AB37" s="7">
+      <c r="AB37">
         <v>3.0235288007063831E-4</v>
       </c>
-      <c r="AC37" s="7">
+      <c r="AC37">
         <v>4.460781745478295E-5</v>
       </c>
-      <c r="AD37" s="7">
+      <c r="AD37">
         <v>6.7780245105495371</v>
       </c>
-      <c r="AE37" s="7">
+      <c r="AE37">
         <v>8.1038648058789092E-5</v>
       </c>
-      <c r="AF37" s="7">
+      <c r="AF37">
         <v>2.0144298629850625E-4</v>
       </c>
-      <c r="AG37" s="7">
+      <c r="AG37">
         <v>4.032627738427704E-4</v>
       </c>
-      <c r="AH37" s="7">
+      <c r="AH37">
         <v>2.0144298629850625E-4</v>
       </c>
-      <c r="AI37" s="7">
+      <c r="AI37">
         <v>4.032627738427704E-4</v>
       </c>
     </row>
-    <row r="38" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>900</v>
       </c>
@@ -6781,11 +6817,11 @@
       <c r="C38">
         <v>13000</v>
       </c>
-      <c r="D38" s="11">
+      <c r="D38" s="10">
         <f t="shared" si="3"/>
         <v>1008000000.0000001</v>
       </c>
-      <c r="E38" s="11">
+      <c r="E38" s="10">
         <f t="shared" si="4"/>
         <v>1072372649.481904</v>
       </c>
@@ -6807,62 +6843,62 @@
         <f t="shared" si="2"/>
         <v>3482.7756791810521</v>
       </c>
-      <c r="Q38" s="8" t="s">
+      <c r="Q38" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="R38" s="8">
+      <c r="R38" s="7">
         <v>-3.8402806153825454E-3</v>
       </c>
-      <c r="S38" s="8">
+      <c r="S38" s="7">
         <v>1.332711165910458E-3</v>
       </c>
-      <c r="T38" s="8">
+      <c r="T38" s="7">
         <v>-2.881555068805183</v>
       </c>
-      <c r="U38" s="8">
+      <c r="U38" s="7">
         <v>1.8132015569115364E-2</v>
       </c>
-      <c r="V38" s="8">
+      <c r="V38" s="7">
         <v>-6.8550827252880355E-3</v>
       </c>
-      <c r="W38" s="8">
+      <c r="W38" s="7">
         <v>-8.2547850547705533E-4</v>
       </c>
-      <c r="X38" s="8">
+      <c r="X38" s="7">
         <v>-6.8550827252880355E-3</v>
       </c>
-      <c r="Y38" s="8">
+      <c r="Y38" s="7">
         <v>-8.2547850547705533E-4</v>
       </c>
-      <c r="AA38" s="8" t="s">
+      <c r="AA38" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="AB38" s="8">
+      <c r="AB38" s="7">
         <v>-1.9462705162655004E-2</v>
       </c>
-      <c r="AC38" s="8">
+      <c r="AC38" s="7">
         <v>6.8839642692857302E-3</v>
       </c>
-      <c r="AD38" s="8">
+      <c r="AD38" s="7">
         <v>-2.8272524959915901</v>
       </c>
-      <c r="AE38" s="8">
+      <c r="AE38" s="7">
         <v>1.9811054120046259E-2</v>
       </c>
-      <c r="AF38" s="8">
+      <c r="AF38" s="7">
         <v>-3.5035314242866634E-2</v>
       </c>
-      <c r="AG38" s="8">
+      <c r="AG38" s="7">
         <v>-3.8900960824433759E-3</v>
       </c>
-      <c r="AH38" s="8">
+      <c r="AH38" s="7">
         <v>-3.5035314242866634E-2</v>
       </c>
-      <c r="AI38" s="8">
+      <c r="AI38" s="7">
         <v>-3.8900960824433759E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>950</v>
       </c>
@@ -6873,11 +6909,11 @@
       <c r="C39">
         <v>13000</v>
       </c>
-      <c r="D39" s="11">
+      <c r="D39" s="10">
         <f t="shared" si="3"/>
         <v>1064000000</v>
       </c>
-      <c r="E39" s="11">
+      <c r="E39" s="10">
         <f t="shared" si="4"/>
         <v>1132524230.7250886</v>
       </c>
@@ -6900,7 +6936,7 @@
         <v>3679.305051226967</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>1000</v>
       </c>
@@ -6911,11 +6947,11 @@
       <c r="C40">
         <v>13000</v>
       </c>
-      <c r="D40" s="11">
+      <c r="D40" s="10">
         <f t="shared" si="3"/>
         <v>1120000000</v>
       </c>
-      <c r="E40" s="11">
+      <c r="E40" s="10">
         <f t="shared" si="4"/>
         <v>1192675811.9682727</v>
       </c>
@@ -6938,7 +6974,7 @@
         <v>3875.8344232728818</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.2">
       <c r="Q42" t="s">
         <v>99</v>
       </c>
@@ -6946,941 +6982,941 @@
         <v>99</v>
       </c>
     </row>
-    <row r="43" spans="1:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="Q44" s="9" t="s">
+    <row r="43" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Q44" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="R44" s="9" t="s">
+      <c r="R44" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="S44" s="9" t="s">
+      <c r="S44" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="AA44" s="9" t="s">
+      <c r="AA44" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="AB44" s="9" t="s">
+      <c r="AB44" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="AC44" s="9" t="s">
+      <c r="AC44" s="8" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="Q45" s="7">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Q45">
         <v>1</v>
       </c>
-      <c r="R45" s="7">
+      <c r="R45">
         <v>49.795768347770696</v>
       </c>
-      <c r="S45" s="7">
+      <c r="S45">
         <v>6.2042316522293106</v>
       </c>
-      <c r="AA45" s="7">
+      <c r="AA45">
         <v>1</v>
       </c>
-      <c r="AB45" s="7">
+      <c r="AB45">
         <v>141.77635440049869</v>
       </c>
-      <c r="AC45" s="7">
+      <c r="AC45">
         <v>29.22364559950131</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="Q46" s="7">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Q46">
         <v>2</v>
       </c>
-      <c r="R46" s="7">
+      <c r="R46">
         <v>109.94734959095501</v>
       </c>
-      <c r="S46" s="7">
+      <c r="S46">
         <v>2.0526504090450004</v>
       </c>
-      <c r="AA46" s="7">
+      <c r="AA46">
         <v>2</v>
       </c>
-      <c r="AB46" s="7">
+      <c r="AB46">
         <v>338.30572644641359</v>
       </c>
-      <c r="AC46" s="7">
+      <c r="AC46">
         <v>3.6942735535864131</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="Q47" s="7">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Q47">
         <v>3</v>
       </c>
-      <c r="R47" s="7">
+      <c r="R47">
         <v>170.09893083413934</v>
       </c>
-      <c r="S47" s="7">
+      <c r="S47">
         <v>-2.0989308341393098</v>
       </c>
-      <c r="AA47" s="7">
+      <c r="AA47">
         <v>3</v>
       </c>
-      <c r="AB47" s="7">
+      <c r="AB47">
         <v>534.83509849232848</v>
       </c>
-      <c r="AC47" s="7">
+      <c r="AC47">
         <v>-21.835098492328484</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="Q48" s="7">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.2">
+      <c r="Q48">
         <v>4</v>
       </c>
-      <c r="R48" s="7">
+      <c r="R48">
         <v>230.25051207732363</v>
       </c>
-      <c r="S48" s="7">
+      <c r="S48">
         <v>-6.2505120773236058</v>
       </c>
-      <c r="AA48" s="7">
+      <c r="AA48">
         <v>4</v>
       </c>
-      <c r="AB48" s="7">
+      <c r="AB48">
         <v>731.36447053824338</v>
       </c>
-      <c r="AC48" s="7">
+      <c r="AC48">
         <v>-47.364470538243381</v>
       </c>
     </row>
-    <row r="49" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q49" s="7">
+    <row r="49" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q49">
         <v>5</v>
       </c>
-      <c r="R49" s="7">
+      <c r="R49">
         <v>42.400185848833345</v>
       </c>
-      <c r="S49" s="7">
+      <c r="S49">
         <v>-15.400185848833345</v>
       </c>
-      <c r="AA49" s="7">
+      <c r="AA49">
         <v>5</v>
       </c>
-      <c r="AB49" s="7">
+      <c r="AB49">
         <v>177.84036202122036</v>
       </c>
-      <c r="AC49" s="7">
+      <c r="AC49">
         <v>-51.840362021220358</v>
       </c>
     </row>
-    <row r="50" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q50" s="7">
+    <row r="50" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q50">
         <v>6</v>
       </c>
-      <c r="R50" s="7">
+      <c r="R50">
         <v>59.057546808484389</v>
       </c>
-      <c r="S50" s="7">
+      <c r="S50">
         <v>-5.0575468084843891</v>
       </c>
-      <c r="AA50" s="7">
+      <c r="AA50">
         <v>6</v>
       </c>
-      <c r="AB50" s="7">
+      <c r="AB50">
         <v>248.89328883782036</v>
       </c>
-      <c r="AC50" s="7">
+      <c r="AC50">
         <v>3.1067111621796357</v>
       </c>
     </row>
-    <row r="51" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q51" s="7">
+    <row r="51" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q51">
         <v>7</v>
       </c>
-      <c r="R51" s="7">
+      <c r="R51">
         <v>75.714907768135433</v>
       </c>
-      <c r="S51" s="7">
+      <c r="S51">
         <v>5.2850922318645672</v>
       </c>
-      <c r="AA51" s="7">
+      <c r="AA51">
         <v>7</v>
       </c>
-      <c r="AB51" s="7">
+      <c r="AB51">
         <v>319.94621565442037</v>
       </c>
-      <c r="AC51" s="7">
+      <c r="AC51">
         <v>58.053784345579629</v>
       </c>
     </row>
-    <row r="52" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q52" s="7">
+    <row r="52" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q52">
         <v>8</v>
       </c>
-      <c r="R52" s="7">
+      <c r="R52">
         <v>92.372268727786476</v>
       </c>
-      <c r="S52" s="7">
+      <c r="S52">
         <v>15.627731272213524</v>
       </c>
-      <c r="AA52" s="7">
+      <c r="AA52">
         <v>8</v>
       </c>
-      <c r="AB52" s="7">
+      <c r="AB52">
         <v>390.99914247102038</v>
       </c>
-      <c r="AC52" s="7">
+      <c r="AC52">
         <v>113.00085752897962</v>
       </c>
     </row>
-    <row r="53" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q53" s="7">
+    <row r="53" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q53">
         <v>9</v>
       </c>
-      <c r="R53" s="7">
+      <c r="R53">
         <v>40.511952019317427</v>
       </c>
-      <c r="S53" s="7">
+      <c r="S53">
         <v>-21.011952019317427</v>
       </c>
-      <c r="AA53" s="7">
+      <c r="AA53">
         <v>9</v>
       </c>
-      <c r="AB53" s="7">
+      <c r="AB53">
         <v>193.04807607815115</v>
       </c>
-      <c r="AC53" s="7">
+      <c r="AC53">
         <v>-113.54807607815115</v>
       </c>
     </row>
-    <row r="54" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q54" s="7">
+    <row r="54" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q54">
         <v>10</v>
       </c>
-      <c r="R54" s="7">
+      <c r="R54">
         <v>46.064405672534441</v>
       </c>
-      <c r="S54" s="7">
+      <c r="S54">
         <v>-7.0644056725344413</v>
       </c>
-      <c r="AA54" s="7">
+      <c r="AA54">
         <v>10</v>
       </c>
-      <c r="AB54" s="7">
+      <c r="AB54">
         <v>211.18924888238945</v>
       </c>
-      <c r="AC54" s="7">
+      <c r="AC54">
         <v>-52.18924888238945</v>
       </c>
     </row>
-    <row r="55" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="Q55" s="7">
+    <row r="55" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="Q55">
         <v>11</v>
       </c>
-      <c r="R55" s="7">
+      <c r="R55">
         <v>51.616859325751456</v>
       </c>
-      <c r="S55" s="7">
+      <c r="S55">
         <v>6.8831406742485441</v>
       </c>
-      <c r="AA55" s="7">
+      <c r="AA55">
         <v>11</v>
       </c>
-      <c r="AB55" s="7">
+      <c r="AB55">
         <v>229.33042168662774</v>
       </c>
-      <c r="AC55" s="7">
+      <c r="AC55">
         <v>9.1695783133722557</v>
       </c>
     </row>
-    <row r="56" spans="17:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="Q56" s="8">
+    <row r="56" spans="17:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="Q56" s="7">
         <v>12</v>
       </c>
-      <c r="R56" s="8">
+      <c r="R56" s="7">
         <v>57.16931297896847</v>
       </c>
-      <c r="S56" s="8">
+      <c r="S56" s="7">
         <v>20.83068702103153</v>
       </c>
-      <c r="AA56" s="8">
+      <c r="AA56" s="7">
         <v>12</v>
       </c>
-      <c r="AB56" s="8">
+      <c r="AB56" s="7">
         <v>247.47159449086604</v>
       </c>
-      <c r="AC56" s="8">
+      <c r="AC56" s="7">
         <v>70.528405509133961</v>
       </c>
     </row>
-    <row r="57" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA57" s="7">
+    <row r="57" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA57">
         <v>13</v>
       </c>
-      <c r="AB57" s="7">
+      <c r="AB57">
         <v>832.73378974792229</v>
       </c>
-      <c r="AC57" s="7">
+      <c r="AC57">
         <v>22.266210252077713</v>
       </c>
     </row>
-    <row r="58" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA58" s="7">
+    <row r="58" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA58">
         <v>14</v>
       </c>
-      <c r="AB58" s="7">
+      <c r="AB58">
         <v>1030.1196596272707</v>
       </c>
-      <c r="AC58" s="7">
+      <c r="AC58">
         <v>-4.1196596272707211</v>
       </c>
     </row>
-    <row r="59" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA59" s="7">
+    <row r="59" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA59">
         <v>15</v>
       </c>
-      <c r="AB59" s="7">
+      <c r="AB59">
         <v>1227.5055295066195</v>
       </c>
-      <c r="AC59" s="7">
+      <c r="AC59">
         <v>-30.505529506619496</v>
       </c>
     </row>
-    <row r="60" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA60" s="7">
+    <row r="60" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA60">
         <v>16</v>
       </c>
-      <c r="AB60" s="7">
+      <c r="AB60">
         <v>1424.8913993859678</v>
       </c>
-      <c r="AC60" s="7">
+      <c r="AC60">
         <v>-56.891399385967816</v>
       </c>
     </row>
-    <row r="61" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA61" s="7">
+    <row r="61" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA61">
         <v>17</v>
       </c>
-      <c r="AB61" s="7">
+      <c r="AB61">
         <v>633.10786470750327</v>
       </c>
-      <c r="AC61" s="7">
+      <c r="AC61">
         <v>-3.1078647075032677</v>
       </c>
     </row>
-    <row r="62" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA62" s="7">
+    <row r="62" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA62">
         <v>18</v>
       </c>
-      <c r="AB62" s="7">
+      <c r="AB62">
         <v>687.76856713563052</v>
       </c>
-      <c r="AC62" s="7">
+      <c r="AC62">
         <v>68.231432864369481</v>
       </c>
     </row>
-    <row r="63" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA63" s="7">
+    <row r="63" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA63">
         <v>19</v>
       </c>
-      <c r="AB63" s="7">
+      <c r="AB63">
         <v>742.42926956375777</v>
       </c>
-      <c r="AC63" s="7">
+      <c r="AC63">
         <v>139.57073043624223</v>
       </c>
     </row>
-    <row r="64" spans="17:29" x14ac:dyDescent="0.25">
-      <c r="AA64" s="7">
+    <row r="64" spans="17:29" x14ac:dyDescent="0.2">
+      <c r="AA64">
         <v>20</v>
       </c>
-      <c r="AB64" s="7">
+      <c r="AB64">
         <v>797.08997199188514</v>
       </c>
-      <c r="AC64" s="7">
+      <c r="AC64">
         <v>210.91002800811486</v>
       </c>
     </row>
-    <row r="65" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA65" s="7">
+    <row r="65" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA65">
         <v>21</v>
       </c>
-      <c r="AB65" s="7">
+      <c r="AB65">
         <v>582.13954342058764</v>
       </c>
-      <c r="AC65" s="7">
+      <c r="AC65">
         <v>-184.63954342058764</v>
       </c>
     </row>
-    <row r="66" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA66" s="7">
+    <row r="66" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA66">
         <v>22</v>
       </c>
-      <c r="AB66" s="7">
+      <c r="AB66">
         <v>600.3597775632968</v>
       </c>
-      <c r="AC66" s="7">
+      <c r="AC66">
         <v>-123.3597775632968</v>
       </c>
     </row>
-    <row r="67" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA67" s="7">
+    <row r="67" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA67">
         <v>23</v>
       </c>
-      <c r="AB67" s="7">
+      <c r="AB67">
         <v>618.58001170600585</v>
       </c>
-      <c r="AC67" s="7">
+      <c r="AC67">
         <v>-62.080011706005848</v>
       </c>
     </row>
-    <row r="68" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA68" s="7">
+    <row r="68" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA68">
         <v>24</v>
       </c>
-      <c r="AB68" s="7">
+      <c r="AB68">
         <v>636.80024584871501</v>
       </c>
-      <c r="AC68" s="7">
+      <c r="AC68">
         <v>-0.80024584871500792</v>
       </c>
     </row>
-    <row r="69" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA69" s="7">
+    <row r="69" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA69">
         <v>25</v>
       </c>
-      <c r="AB69" s="7">
+      <c r="AB69">
         <v>1622.2772692653166</v>
       </c>
-      <c r="AC69" s="7">
+      <c r="AC69">
         <v>-83.27726926531659</v>
       </c>
     </row>
-    <row r="70" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA70" s="7">
+    <row r="70" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA70">
         <v>26</v>
       </c>
-      <c r="AB70" s="7">
+      <c r="AB70">
         <v>1819.6631391446649</v>
       </c>
-      <c r="AC70" s="7">
+      <c r="AC70">
         <v>-109.66313914466491</v>
       </c>
     </row>
-    <row r="71" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA71" s="7">
+    <row r="71" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA71">
         <v>27</v>
       </c>
-      <c r="AB71" s="7">
+      <c r="AB71">
         <v>2017.0490090240137</v>
       </c>
-      <c r="AC71" s="7">
+      <c r="AC71">
         <v>-136.04900902401369</v>
       </c>
     </row>
-    <row r="72" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA72" s="7">
+    <row r="72" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA72">
         <v>28</v>
       </c>
-      <c r="AB72" s="7">
+      <c r="AB72">
         <v>2214.434878903362</v>
       </c>
-      <c r="AC72" s="7">
+      <c r="AC72">
         <v>-162.43487890336201</v>
       </c>
     </row>
-    <row r="73" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA73" s="7">
+    <row r="73" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA73">
         <v>29</v>
       </c>
-      <c r="AB73" s="7">
+      <c r="AB73">
         <v>851.7506744200125</v>
       </c>
-      <c r="AC73" s="7">
+      <c r="AC73">
         <v>282.2493255799875</v>
       </c>
     </row>
-    <row r="74" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA74" s="7">
+    <row r="74" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA74">
         <v>30</v>
       </c>
-      <c r="AB74" s="7">
+      <c r="AB74">
         <v>906.41137684813975</v>
       </c>
-      <c r="AC74" s="7">
+      <c r="AC74">
         <v>353.58862315186025</v>
       </c>
     </row>
-    <row r="75" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA75" s="7">
+    <row r="75" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA75">
         <v>31</v>
       </c>
-      <c r="AB75" s="7">
+      <c r="AB75">
         <v>961.072079276267</v>
       </c>
-      <c r="AC75" s="7">
+      <c r="AC75">
         <v>424.927920723733</v>
       </c>
     </row>
-    <row r="76" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA76" s="7">
+    <row r="76" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA76">
         <v>32</v>
       </c>
-      <c r="AB76" s="7">
+      <c r="AB76">
         <v>1015.7327817043943</v>
       </c>
-      <c r="AC76" s="7">
+      <c r="AC76">
         <v>496.26721829560574</v>
       </c>
     </row>
-    <row r="77" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA77" s="7">
+    <row r="77" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA77">
         <v>33</v>
       </c>
-      <c r="AB77" s="7">
+      <c r="AB77">
         <v>655.02047999142405</v>
       </c>
-      <c r="AC77" s="7">
+      <c r="AC77">
         <v>60.479520008575946</v>
       </c>
     </row>
-    <row r="78" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA78" s="7">
+    <row r="78" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA78">
         <v>34</v>
       </c>
-      <c r="AB78" s="7">
+      <c r="AB78">
         <v>673.2407141341331</v>
       </c>
-      <c r="AC78" s="7">
+      <c r="AC78">
         <v>121.7592858658669</v>
       </c>
     </row>
-    <row r="79" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA79" s="7">
+    <row r="79" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA79">
         <v>35</v>
       </c>
-      <c r="AB79" s="7">
+      <c r="AB79">
         <v>691.46094827684226</v>
       </c>
-      <c r="AC79" s="7">
+      <c r="AC79">
         <v>183.03905172315774</v>
       </c>
     </row>
-    <row r="80" spans="27:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="AA80" s="8">
+    <row r="80" spans="27:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AA80" s="7">
         <v>36</v>
       </c>
-      <c r="AB80" s="8">
+      <c r="AB80" s="7">
         <v>709.68118241955142</v>
       </c>
-      <c r="AC80" s="8">
+      <c r="AC80" s="7">
         <v>244.31881758044858</v>
       </c>
     </row>
-    <row r="81" spans="27:29" x14ac:dyDescent="0.25">
+    <row r="81" spans="27:29" x14ac:dyDescent="0.2">
       <c r="AA81" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="82" spans="27:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="83" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA83" s="9" t="s">
+    <row r="82" spans="27:29" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA83" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="AB83" s="9" t="s">
+      <c r="AB83" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="AC83" s="9" t="s">
+      <c r="AC83" s="8" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="84" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA84" s="7">
+    <row r="84" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA84">
         <v>1</v>
       </c>
-      <c r="AB84" s="7">
+      <c r="AB84">
         <v>196.57832677676012</v>
       </c>
-      <c r="AC84" s="7">
+      <c r="AC84">
         <v>-25.578326776760122</v>
       </c>
     </row>
-    <row r="85" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA85" s="7">
+    <row r="85" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA85">
         <v>2</v>
       </c>
-      <c r="AB85" s="7">
+      <c r="AB85">
         <v>393.05682104494429</v>
       </c>
-      <c r="AC85" s="7">
+      <c r="AC85">
         <v>-51.056821044944286</v>
       </c>
     </row>
-    <row r="86" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA86" s="7">
+    <row r="86" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA86">
         <v>3</v>
       </c>
-      <c r="AB86" s="7">
+      <c r="AB86">
         <v>589.53531531312842</v>
       </c>
-      <c r="AC86" s="7">
+      <c r="AC86">
         <v>-76.535315313128422</v>
       </c>
     </row>
-    <row r="87" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA87" s="7">
+    <row r="87" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA87">
         <v>4</v>
       </c>
-      <c r="AB87" s="7">
+      <c r="AB87">
         <v>786.01380958131267</v>
       </c>
-      <c r="AC87" s="7">
+      <c r="AC87">
         <v>-102.01380958131267</v>
       </c>
     </row>
-    <row r="88" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA88" s="7">
+    <row r="88" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA88">
         <v>5</v>
       </c>
-      <c r="AB88" s="7">
+      <c r="AB88">
         <v>71.070625834674814</v>
       </c>
-      <c r="AC88" s="7">
+      <c r="AC88">
         <v>54.929374165325186</v>
       </c>
     </row>
-    <row r="89" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA89" s="7">
+    <row r="89" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA89">
         <v>6</v>
       </c>
-      <c r="AB89" s="7">
+      <c r="AB89">
         <v>142.10515837778755</v>
       </c>
-      <c r="AC89" s="7">
+      <c r="AC89">
         <v>109.89484162221245</v>
       </c>
     </row>
-    <row r="90" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA90" s="7">
+    <row r="90" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA90">
         <v>7</v>
       </c>
-      <c r="AB90" s="7">
+      <c r="AB90">
         <v>213.13969092090028</v>
       </c>
-      <c r="AC90" s="7">
+      <c r="AC90">
         <v>164.86030907909972</v>
       </c>
     </row>
-    <row r="91" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA91" s="7">
+    <row r="91" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA91">
         <v>8</v>
       </c>
-      <c r="AB91" s="7">
+      <c r="AB91">
         <v>284.17422346401298</v>
       </c>
-      <c r="AC91" s="7">
+      <c r="AC91">
         <v>219.82577653598702</v>
       </c>
     </row>
-    <row r="92" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA92" s="7">
+    <row r="92" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA92">
         <v>9</v>
       </c>
-      <c r="AB92" s="7">
+      <c r="AB92">
         <v>18.145691702470163</v>
       </c>
-      <c r="AC92" s="7">
+      <c r="AC92">
         <v>61.35430829752984</v>
       </c>
     </row>
-    <row r="93" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA93" s="7">
+    <row r="93" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA93">
         <v>10</v>
       </c>
-      <c r="AB93" s="7">
+      <c r="AB93">
         <v>36.282168096456395</v>
       </c>
-      <c r="AC93" s="7">
+      <c r="AC93">
         <v>122.71783190354361</v>
       </c>
     </row>
-    <row r="94" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA94" s="7">
+    <row r="94" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA94">
         <v>11</v>
       </c>
-      <c r="AB94" s="7">
+      <c r="AB94">
         <v>54.418644490442624</v>
       </c>
-      <c r="AC94" s="7">
+      <c r="AC94">
         <v>184.08135550955737</v>
       </c>
     </row>
-    <row r="95" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA95" s="7">
+    <row r="95" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA95">
         <v>12</v>
       </c>
-      <c r="AB95" s="7">
+      <c r="AB95">
         <v>72.555120884428845</v>
       </c>
-      <c r="AC95" s="7">
+      <c r="AC95">
         <v>245.44487911557115</v>
       </c>
     </row>
-    <row r="96" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA96" s="7">
+    <row r="96" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA96">
         <v>13</v>
       </c>
-      <c r="AB96" s="7">
+      <c r="AB96">
         <v>982.49230384949681</v>
       </c>
-      <c r="AC96" s="7">
+      <c r="AC96">
         <v>-127.49230384949681</v>
       </c>
     </row>
-    <row r="97" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA97" s="7">
+    <row r="97" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA97">
         <v>14</v>
       </c>
-      <c r="AB97" s="7">
+      <c r="AB97">
         <v>1178.9707981176807</v>
       </c>
-      <c r="AC97" s="7">
+      <c r="AC97">
         <v>-152.97079811768072</v>
       </c>
     </row>
-    <row r="98" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA98" s="7">
+    <row r="98" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA98">
         <v>15</v>
       </c>
-      <c r="AB98" s="7">
+      <c r="AB98">
         <v>1375.449292385865</v>
       </c>
-      <c r="AC98" s="7">
+      <c r="AC98">
         <v>-178.44929238586496</v>
       </c>
     </row>
-    <row r="99" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA99" s="7">
+    <row r="99" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA99">
         <v>16</v>
       </c>
-      <c r="AB99" s="7">
+      <c r="AB99">
         <v>1571.9277866540492</v>
       </c>
-      <c r="AC99" s="7">
+      <c r="AC99">
         <v>-203.92778665404921</v>
       </c>
     </row>
-    <row r="100" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA100" s="7">
+    <row r="100" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA100">
         <v>17</v>
       </c>
-      <c r="AB100" s="7">
+      <c r="AB100">
         <v>272.07479183524526</v>
       </c>
-      <c r="AC100" s="7">
+      <c r="AC100">
         <v>357.92520816475474</v>
       </c>
     </row>
-    <row r="101" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA101" s="7">
+    <row r="101" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA101">
         <v>18</v>
       </c>
-      <c r="AB101" s="7">
+      <c r="AB101">
         <v>326.48422101720394</v>
       </c>
-      <c r="AC101" s="7">
+      <c r="AC101">
         <v>429.51577898279606</v>
       </c>
     </row>
-    <row r="102" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA102" s="7">
+    <row r="102" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA102">
         <v>19</v>
       </c>
-      <c r="AB102" s="7">
+      <c r="AB102">
         <v>380.89365019916261</v>
       </c>
-      <c r="AC102" s="7">
+      <c r="AC102">
         <v>501.10634980083739</v>
       </c>
     </row>
-    <row r="103" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA103" s="7">
+    <row r="103" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA103">
         <v>20</v>
       </c>
-      <c r="AB103" s="7">
+      <c r="AB103">
         <v>435.30307938112128</v>
       </c>
-      <c r="AC103" s="7">
+      <c r="AC103">
         <v>572.69692061887872</v>
       </c>
     </row>
-    <row r="104" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA104" s="7">
+    <row r="104" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA104">
         <v>21</v>
       </c>
-      <c r="AB104" s="7">
+      <c r="AB104">
         <v>90.691597278415074</v>
       </c>
-      <c r="AC104" s="7">
+      <c r="AC104">
         <v>306.80840272158491</v>
       </c>
     </row>
-    <row r="105" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA105" s="7">
+    <row r="105" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA105">
         <v>22</v>
       </c>
-      <c r="AB105" s="7">
+      <c r="AB105">
         <v>108.8280736724013</v>
       </c>
-      <c r="AC105" s="7">
+      <c r="AC105">
         <v>368.17192632759873</v>
       </c>
     </row>
-    <row r="106" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA106" s="7">
+    <row r="106" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA106">
         <v>23</v>
       </c>
-      <c r="AB106" s="7">
+      <c r="AB106">
         <v>126.96455006638755</v>
       </c>
-      <c r="AC106" s="7">
+      <c r="AC106">
         <v>429.53544993361243</v>
       </c>
     </row>
-    <row r="107" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA107" s="7">
+    <row r="107" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA107">
         <v>24</v>
       </c>
-      <c r="AB107" s="7">
+      <c r="AB107">
         <v>145.10102646037376</v>
       </c>
-      <c r="AC107" s="7">
+      <c r="AC107">
         <v>490.89897353962624</v>
       </c>
     </row>
-    <row r="108" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA108" s="7">
+    <row r="108" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA108">
         <v>25</v>
       </c>
-      <c r="AB108" s="7">
+      <c r="AB108">
         <v>1768.4062809222332</v>
       </c>
-      <c r="AC108" s="7">
+      <c r="AC108">
         <v>-229.40628092223324</v>
       </c>
     </row>
-    <row r="109" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA109" s="7">
+    <row r="109" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA109">
         <v>26</v>
       </c>
-      <c r="AB109" s="7">
+      <c r="AB109">
         <v>1964.8847751904175</v>
       </c>
-      <c r="AC109" s="7">
+      <c r="AC109">
         <v>-254.88477519041749</v>
       </c>
     </row>
-    <row r="110" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA110" s="7">
+    <row r="110" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA110">
         <v>27</v>
       </c>
-      <c r="AB110" s="7">
+      <c r="AB110">
         <v>2161.3632694586017</v>
       </c>
-      <c r="AC110" s="7">
+      <c r="AC110">
         <v>-280.36326945860174</v>
       </c>
     </row>
-    <row r="111" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA111" s="7">
+    <row r="111" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA111">
         <v>28</v>
       </c>
-      <c r="AB111" s="7">
+      <c r="AB111">
         <v>2357.8417637267858</v>
       </c>
-      <c r="AC111" s="7">
+      <c r="AC111">
         <v>-305.84176372678576</v>
       </c>
     </row>
-    <row r="112" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA112" s="7">
+    <row r="112" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA112">
         <v>29</v>
       </c>
-      <c r="AB112" s="7">
+      <c r="AB112">
         <v>489.71250856308001</v>
       </c>
-      <c r="AC112" s="7">
+      <c r="AC112">
         <v>644.28749143691994</v>
       </c>
     </row>
-    <row r="113" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA113" s="7">
+    <row r="113" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA113">
         <v>30</v>
       </c>
-      <c r="AB113" s="7">
+      <c r="AB113">
         <v>544.12193774503874</v>
       </c>
-      <c r="AC113" s="7">
+      <c r="AC113">
         <v>715.87806225496126</v>
       </c>
     </row>
-    <row r="114" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA114" s="7">
+    <row r="114" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA114">
         <v>31</v>
       </c>
-      <c r="AB114" s="7">
+      <c r="AB114">
         <v>598.53136692699741</v>
       </c>
-      <c r="AC114" s="7">
+      <c r="AC114">
         <v>787.46863307300259</v>
       </c>
     </row>
-    <row r="115" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA115" s="7">
+    <row r="115" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA115">
         <v>32</v>
       </c>
-      <c r="AB115" s="7">
+      <c r="AB115">
         <v>652.94079610895608</v>
       </c>
-      <c r="AC115" s="7">
+      <c r="AC115">
         <v>859.05920389104392</v>
       </c>
     </row>
-    <row r="116" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA116" s="7">
+    <row r="116" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA116">
         <v>33</v>
       </c>
-      <c r="AB116" s="7">
+      <c r="AB116">
         <v>163.23750285436</v>
       </c>
-      <c r="AC116" s="7">
+      <c r="AC116">
         <v>552.26249714564005</v>
       </c>
     </row>
-    <row r="117" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA117" s="7">
+    <row r="117" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA117">
         <v>34</v>
       </c>
-      <c r="AB117" s="7">
+      <c r="AB117">
         <v>181.37397924834622</v>
       </c>
-      <c r="AC117" s="7">
+      <c r="AC117">
         <v>613.62602075165375</v>
       </c>
     </row>
-    <row r="118" spans="27:29" x14ac:dyDescent="0.25">
-      <c r="AA118" s="7">
+    <row r="118" spans="27:29" x14ac:dyDescent="0.2">
+      <c r="AA118">
         <v>35</v>
       </c>
-      <c r="AB118" s="7">
+      <c r="AB118">
         <v>199.51045564233246</v>
       </c>
-      <c r="AC118" s="7">
+      <c r="AC118">
         <v>674.98954435766757</v>
       </c>
     </row>
-    <row r="119" spans="27:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="AA119" s="8">
+    <row r="119" spans="27:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="AA119" s="7">
         <v>36</v>
       </c>
-      <c r="AB119" s="8">
+      <c r="AB119" s="7">
         <v>217.64693203631867</v>
       </c>
-      <c r="AC119" s="8">
+      <c r="AC119" s="7">
         <v>736.35306796368127</v>
       </c>
     </row>
@@ -7896,14 +7932,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DDCD6FE-4E00-4CD6-871A-4D2AE5966951}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:V19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -7920,7 +7956,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="L2" t="s">
         <v>11</v>
       </c>
@@ -7928,7 +7964,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="M4" t="s">
         <v>49</v>
       </c>
@@ -7948,7 +7984,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>21</v>
       </c>
@@ -7983,7 +8019,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>24</v>
       </c>
@@ -8033,7 +8069,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>37</v>
       </c>
@@ -8106,7 +8142,7 @@
         <v>125475000</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>38</v>
       </c>
@@ -8179,7 +8215,7 @@
         <v>110040000</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>39</v>
       </c>
@@ -8252,7 +8288,7 @@
         <v>123182500.00000001</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>40</v>
       </c>
@@ -8325,7 +8361,7 @@
         <v>112525000</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>41</v>
       </c>
@@ -8398,7 +8434,7 @@
         <v>161985250</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>42</v>
       </c>
@@ -8471,7 +8507,7 @@
         <v>110313000</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>43</v>
       </c>
@@ -8544,7 +8580,7 @@
         <v>75075000</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>44</v>
       </c>
@@ -8617,7 +8653,7 @@
         <v>67725000</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>45</v>
       </c>
@@ -8690,7 +8726,7 @@
         <v>158891250</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>46</v>
       </c>
@@ -8763,7 +8799,7 @@
         <v>106750000</v>
       </c>
     </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>47</v>
       </c>
@@ -8836,7 +8872,7 @@
         <v>82285000</v>
       </c>
     </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>41</v>
       </c>
@@ -8909,7 +8945,7 @@
         <v>269057250</v>
       </c>
     </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>48</v>
       </c>
@@ -8991,9 +9027,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{220A59A8-D123-4429-B71D-A74BAF1E63EB}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>54</v>
       </c>

</xml_diff>